<commit_message>
Added VISTIT to the output varaibles list and test data upated
</commit_message>
<xml_diff>
--- a/rules/CORE-000270/negative/02/data/unit-test-coreid-CG0033-negative2.xlsx
+++ b/rules/CORE-000270/negative/02/data/unit-test-coreid-CG0033-negative2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JanakiRaman\CORE\Rule_Authoring\core-contributor\rules\CORE-000270\negative\02\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7560FB71-43ED-4238-B8C4-4C896D5D7621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3197E3C5-659A-4488-9F11-0DAF0DE40189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9719" uniqueCount="749">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9823" uniqueCount="749">
   <si>
     <t>Product</t>
   </si>
@@ -2286,7 +2286,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2303,6 +2303,12 @@
       <i/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -2753,7 +2759,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="5" max="5" width="9.6328125" bestFit="1" customWidth="1"/>
@@ -3299,7 +3305,528 @@
         <v>12</v>
       </c>
     </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>2</v>
+      </c>
+      <c r="B28" t="s">
+        <v>14</v>
+      </c>
+      <c r="C28" t="s">
+        <v>748</v>
+      </c>
+      <c r="D28">
+        <v>35</v>
+      </c>
+      <c r="E28" t="s">
+        <v>76</v>
+      </c>
+      <c r="F28" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>3</v>
+      </c>
+      <c r="B29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C29" t="s">
+        <v>748</v>
+      </c>
+      <c r="D29">
+        <v>36</v>
+      </c>
+      <c r="E29" t="s">
+        <v>76</v>
+      </c>
+      <c r="F29" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>4</v>
+      </c>
+      <c r="B30" t="s">
+        <v>14</v>
+      </c>
+      <c r="C30" t="s">
+        <v>748</v>
+      </c>
+      <c r="D30">
+        <v>37</v>
+      </c>
+      <c r="E30" t="s">
+        <v>76</v>
+      </c>
+      <c r="F30" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>5</v>
+      </c>
+      <c r="B31" t="s">
+        <v>14</v>
+      </c>
+      <c r="C31" t="s">
+        <v>748</v>
+      </c>
+      <c r="D31">
+        <v>69</v>
+      </c>
+      <c r="E31" t="s">
+        <v>76</v>
+      </c>
+      <c r="F31" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>6</v>
+      </c>
+      <c r="B32" t="s">
+        <v>14</v>
+      </c>
+      <c r="C32" t="s">
+        <v>748</v>
+      </c>
+      <c r="D32">
+        <v>70</v>
+      </c>
+      <c r="E32" t="s">
+        <v>76</v>
+      </c>
+      <c r="F32" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>7</v>
+      </c>
+      <c r="B33" t="s">
+        <v>14</v>
+      </c>
+      <c r="C33" t="s">
+        <v>748</v>
+      </c>
+      <c r="D33">
+        <v>71</v>
+      </c>
+      <c r="E33" t="s">
+        <v>76</v>
+      </c>
+      <c r="F33" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <v>8</v>
+      </c>
+      <c r="B34" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34" t="s">
+        <v>748</v>
+      </c>
+      <c r="D34">
+        <v>102</v>
+      </c>
+      <c r="E34" t="s">
+        <v>76</v>
+      </c>
+      <c r="F34" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <v>9</v>
+      </c>
+      <c r="B35" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35" t="s">
+        <v>748</v>
+      </c>
+      <c r="D35">
+        <v>103</v>
+      </c>
+      <c r="E35" t="s">
+        <v>76</v>
+      </c>
+      <c r="F35" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>10</v>
+      </c>
+      <c r="B36" t="s">
+        <v>14</v>
+      </c>
+      <c r="C36" t="s">
+        <v>748</v>
+      </c>
+      <c r="D36">
+        <v>104</v>
+      </c>
+      <c r="E36" t="s">
+        <v>76</v>
+      </c>
+      <c r="F36" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>11</v>
+      </c>
+      <c r="B37" t="s">
+        <v>14</v>
+      </c>
+      <c r="C37" t="s">
+        <v>748</v>
+      </c>
+      <c r="D37">
+        <v>115</v>
+      </c>
+      <c r="E37" t="s">
+        <v>76</v>
+      </c>
+      <c r="F37" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>12</v>
+      </c>
+      <c r="B38" t="s">
+        <v>14</v>
+      </c>
+      <c r="C38" t="s">
+        <v>748</v>
+      </c>
+      <c r="D38">
+        <v>125</v>
+      </c>
+      <c r="E38" t="s">
+        <v>76</v>
+      </c>
+      <c r="F38" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39">
+        <v>13</v>
+      </c>
+      <c r="B39" t="s">
+        <v>14</v>
+      </c>
+      <c r="C39" t="s">
+        <v>748</v>
+      </c>
+      <c r="D39">
+        <v>156</v>
+      </c>
+      <c r="E39" t="s">
+        <v>76</v>
+      </c>
+      <c r="F39" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40">
+        <v>14</v>
+      </c>
+      <c r="B40" t="s">
+        <v>14</v>
+      </c>
+      <c r="C40" t="s">
+        <v>748</v>
+      </c>
+      <c r="D40">
+        <v>157</v>
+      </c>
+      <c r="E40" t="s">
+        <v>76</v>
+      </c>
+      <c r="F40" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A41">
+        <v>15</v>
+      </c>
+      <c r="B41" t="s">
+        <v>14</v>
+      </c>
+      <c r="C41" t="s">
+        <v>748</v>
+      </c>
+      <c r="D41">
+        <v>158</v>
+      </c>
+      <c r="E41" t="s">
+        <v>76</v>
+      </c>
+      <c r="F41" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A42">
+        <v>16</v>
+      </c>
+      <c r="B42" t="s">
+        <v>14</v>
+      </c>
+      <c r="C42" t="s">
+        <v>748</v>
+      </c>
+      <c r="D42">
+        <v>190</v>
+      </c>
+      <c r="E42" t="s">
+        <v>76</v>
+      </c>
+      <c r="F42" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A43">
+        <v>17</v>
+      </c>
+      <c r="B43" t="s">
+        <v>14</v>
+      </c>
+      <c r="C43" t="s">
+        <v>748</v>
+      </c>
+      <c r="D43">
+        <v>191</v>
+      </c>
+      <c r="E43" t="s">
+        <v>76</v>
+      </c>
+      <c r="F43" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A44">
+        <v>18</v>
+      </c>
+      <c r="B44" t="s">
+        <v>14</v>
+      </c>
+      <c r="C44" t="s">
+        <v>748</v>
+      </c>
+      <c r="D44">
+        <v>192</v>
+      </c>
+      <c r="E44" t="s">
+        <v>76</v>
+      </c>
+      <c r="F44" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A45">
+        <v>19</v>
+      </c>
+      <c r="B45" t="s">
+        <v>14</v>
+      </c>
+      <c r="C45" t="s">
+        <v>748</v>
+      </c>
+      <c r="D45">
+        <v>223</v>
+      </c>
+      <c r="E45" t="s">
+        <v>76</v>
+      </c>
+      <c r="F45" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46">
+        <v>20</v>
+      </c>
+      <c r="B46" t="s">
+        <v>14</v>
+      </c>
+      <c r="C46" t="s">
+        <v>748</v>
+      </c>
+      <c r="D46">
+        <v>224</v>
+      </c>
+      <c r="E46" t="s">
+        <v>76</v>
+      </c>
+      <c r="F46" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A47">
+        <v>21</v>
+      </c>
+      <c r="B47" t="s">
+        <v>14</v>
+      </c>
+      <c r="C47" t="s">
+        <v>748</v>
+      </c>
+      <c r="D47">
+        <v>225</v>
+      </c>
+      <c r="E47" t="s">
+        <v>76</v>
+      </c>
+      <c r="F47" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A48">
+        <v>22</v>
+      </c>
+      <c r="B48" t="s">
+        <v>14</v>
+      </c>
+      <c r="C48" t="s">
+        <v>748</v>
+      </c>
+      <c r="D48">
+        <v>236</v>
+      </c>
+      <c r="E48" t="s">
+        <v>76</v>
+      </c>
+      <c r="F48" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A49">
+        <v>23</v>
+      </c>
+      <c r="B49" t="s">
+        <v>14</v>
+      </c>
+      <c r="C49" t="s">
+        <v>748</v>
+      </c>
+      <c r="D49">
+        <v>246</v>
+      </c>
+      <c r="E49" t="s">
+        <v>76</v>
+      </c>
+      <c r="F49" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A50">
+        <v>24</v>
+      </c>
+      <c r="B50" t="s">
+        <v>10</v>
+      </c>
+      <c r="C50" t="s">
+        <v>748</v>
+      </c>
+      <c r="D50">
+        <v>15</v>
+      </c>
+      <c r="E50" t="s">
+        <v>76</v>
+      </c>
+      <c r="F50" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A51">
+        <v>25</v>
+      </c>
+      <c r="B51" t="s">
+        <v>10</v>
+      </c>
+      <c r="C51" t="s">
+        <v>748</v>
+      </c>
+      <c r="D51">
+        <v>26</v>
+      </c>
+      <c r="E51" t="s">
+        <v>76</v>
+      </c>
+      <c r="F51" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A52">
+        <v>26</v>
+      </c>
+      <c r="B52" t="s">
+        <v>10</v>
+      </c>
+      <c r="C52" t="s">
+        <v>748</v>
+      </c>
+      <c r="D52">
+        <v>27</v>
+      </c>
+      <c r="E52" t="s">
+        <v>76</v>
+      </c>
+      <c r="F52" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A53">
+        <v>27</v>
+      </c>
+      <c r="B53" t="s">
+        <v>10</v>
+      </c>
+      <c r="C53" t="s">
+        <v>748</v>
+      </c>
+      <c r="D53">
+        <v>39</v>
+      </c>
+      <c r="E53" t="s">
+        <v>76</v>
+      </c>
+      <c r="F53" t="s">
+        <v>549</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -23229,7 +23756,7 @@
       <c r="D15" s="5">
         <v>12</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="5" t="s">
         <v>549</v>
       </c>
       <c r="F15" s="4" t="s">
@@ -23614,7 +24141,7 @@
       <c r="D26" s="5">
         <v>12</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="5" t="s">
         <v>549</v>
       </c>
       <c r="F26" s="4" t="s">
@@ -23649,7 +24176,7 @@
       <c r="D27" s="5">
         <v>13</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="5" t="s">
         <v>559</v>
       </c>
       <c r="F27" s="4" t="s">
@@ -24068,7 +24595,7 @@
       <c r="D39" s="5">
         <v>12</v>
       </c>
-      <c r="E39" s="4" t="s">
+      <c r="E39" s="5" t="s">
         <v>549</v>
       </c>
       <c r="F39" s="4" t="s">
@@ -24094,6 +24621,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:L39" xr:uid="{00000000-0001-0000-0600-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -26405,7 +26933,7 @@
       <c r="Q35" s="5">
         <v>12</v>
       </c>
-      <c r="R35" s="4" t="s">
+      <c r="R35" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S35" s="4" t="s">
@@ -26461,7 +26989,7 @@
       <c r="Q36" s="5">
         <v>12</v>
       </c>
-      <c r="R36" s="4" t="s">
+      <c r="R36" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S36" s="4" t="s">
@@ -26517,7 +27045,7 @@
       <c r="Q37" s="5">
         <v>12</v>
       </c>
-      <c r="R37" s="4" t="s">
+      <c r="R37" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S37" s="4" t="s">
@@ -28306,7 +28834,7 @@
       <c r="Q69" s="5">
         <v>12</v>
       </c>
-      <c r="R69" s="4" t="s">
+      <c r="R69" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S69" s="4" t="s">
@@ -28362,7 +28890,7 @@
       <c r="Q70" s="5">
         <v>12</v>
       </c>
-      <c r="R70" s="4" t="s">
+      <c r="R70" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S70" s="4" t="s">
@@ -28418,7 +28946,7 @@
       <c r="Q71" s="5">
         <v>12</v>
       </c>
-      <c r="R71" s="4" t="s">
+      <c r="R71" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S71" s="4" t="s">
@@ -30157,7 +30685,7 @@
       <c r="Q102" s="5">
         <v>12</v>
       </c>
-      <c r="R102" s="4" t="s">
+      <c r="R102" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S102" s="4" t="s">
@@ -30213,7 +30741,7 @@
       <c r="Q103" s="5">
         <v>12</v>
       </c>
-      <c r="R103" s="4" t="s">
+      <c r="R103" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S103" s="4" t="s">
@@ -30269,7 +30797,7 @@
       <c r="Q104" s="5">
         <v>12</v>
       </c>
-      <c r="R104" s="4" t="s">
+      <c r="R104" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S104" s="4" t="s">
@@ -30855,7 +31383,7 @@
       <c r="Q115" s="5">
         <v>12</v>
       </c>
-      <c r="R115" s="4" t="s">
+      <c r="R115" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S115" s="4" t="s">
@@ -31358,7 +31886,7 @@
       <c r="Q125" s="5">
         <v>12</v>
       </c>
-      <c r="R125" s="4" t="s">
+      <c r="R125" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S125" s="4" t="s">
@@ -33097,7 +33625,7 @@
       <c r="Q156" s="5">
         <v>12</v>
       </c>
-      <c r="R156" s="4" t="s">
+      <c r="R156" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S156" s="4" t="s">
@@ -33153,7 +33681,7 @@
       <c r="Q157" s="5">
         <v>12</v>
       </c>
-      <c r="R157" s="4" t="s">
+      <c r="R157" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S157" s="4" t="s">
@@ -33209,7 +33737,7 @@
       <c r="Q158" s="5">
         <v>12</v>
       </c>
-      <c r="R158" s="4" t="s">
+      <c r="R158" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S158" s="4" t="s">
@@ -34998,7 +35526,7 @@
       <c r="Q190" s="5">
         <v>12</v>
       </c>
-      <c r="R190" s="4" t="s">
+      <c r="R190" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S190" s="4" t="s">
@@ -35054,7 +35582,7 @@
       <c r="Q191" s="5">
         <v>12</v>
       </c>
-      <c r="R191" s="4" t="s">
+      <c r="R191" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S191" s="4" t="s">
@@ -35110,7 +35638,7 @@
       <c r="Q192" s="5">
         <v>12</v>
       </c>
-      <c r="R192" s="4" t="s">
+      <c r="R192" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S192" s="4" t="s">
@@ -36849,7 +37377,7 @@
       <c r="Q223" s="5">
         <v>12</v>
       </c>
-      <c r="R223" s="4" t="s">
+      <c r="R223" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S223" s="4" t="s">
@@ -36905,7 +37433,7 @@
       <c r="Q224" s="5">
         <v>12</v>
       </c>
-      <c r="R224" s="4" t="s">
+      <c r="R224" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S224" s="4" t="s">
@@ -36961,7 +37489,7 @@
       <c r="Q225" s="5">
         <v>12</v>
       </c>
-      <c r="R225" s="4" t="s">
+      <c r="R225" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S225" s="4" t="s">
@@ -37544,7 +38072,7 @@
       <c r="Q236" s="5">
         <v>12</v>
       </c>
-      <c r="R236" s="4" t="s">
+      <c r="R236" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S236" s="4" t="s">
@@ -38044,7 +38572,7 @@
       <c r="Q246" s="5">
         <v>12</v>
       </c>
-      <c r="R246" s="4" t="s">
+      <c r="R246" s="5" t="s">
         <v>549</v>
       </c>
       <c r="S246" s="4" t="s">

</xml_diff>